<commit_message>
PS4 ausgeblendet, WinUAE (Amiga) ergänzt
</commit_message>
<xml_diff>
--- a/docs/emulatoren_mit_downloadanleitungen.xlsx
+++ b/docs/emulatoren_mit_downloadanleitungen.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start hier" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Emulatoren" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Start hier" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Emulatoren" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Emulatoren'!$A$1:$H$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Emulatoren'!$A$1:$H$26</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -222,6 +222,7 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Codex</author>
+    <author>Emulator Hub</author>
   </authors>
   <commentList>
     <comment ref="F2" authorId="0" shapeId="0">
@@ -376,6 +377,16 @@
         <t>Offizielle Quelle, im Browser geprüft am 01.10.2026.
 Primärlink: https://github.com/finalburnneo/FBNeo/releases
 Hinweis: Links in der Beschreibung können auf zusätzliche offizielle Projektseiten verweisen.</t>
+      </text>
+    </comment>
+    <comment ref="F26" authorId="1" shapeId="0">
+      <text>
+        <t>Quelle: https://www.winuae.net/download/; live geprueft am 03.10.2026. Vier verlinkte x86/x64-MSI-/ZIP-Dateien kommen offiziell von https://download.abime.net/winuae/releases/. Die aktuelle stabile Version war 6.0.3. Keine offizielle Hersteller-Pruefsumme oder dedizierte Versions-API gefunden.</t>
+      </text>
+    </comment>
+    <comment ref="G26" authorId="1" shapeId="0">
+      <text>
+        <t>Automatischer Weg im Hub: direct_resolver=winuae, nur aktuelles stabiles x64-ZIP mit eindeutiger Versions-/Dateinamenpruefung. Nach Format-/Quellenaenderung manuell einrichten. CLI fuer eigene .uae-Konfiguration: https://github.com/tonioni/WinUAE/blob/6030/main.cpp und cfgfile.cpp; Endungen: https://www.winuae.net/features/ und od-win32/win32gui.cpp am stabilen Tag 6030.</t>
       </text>
     </comment>
   </commentList>
@@ -804,7 +815,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1783,18 +1794,144 @@
         </is>
       </c>
     </row>
-    <row r="24"/>
-    <row r="25" ht="32" customHeight="1">
-      <c r="A25" s="10" t="inlineStr">
-        <is>
-          <t>Hinweis: Switch und PS4 fehlen, da es keinen empfehlenswerten, aktiv gepflegten Emulator gibt.</t>
+    <row r="24" ht="180" customHeight="1">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>Sony</t>
+        </is>
+      </c>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>PlayStation 4</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>shadPS4</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>Windows/Linux (x64), macOS (Apple Silicon mit Rosetta 2; keine Intel-Macs)</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>Sehr hoch</t>
+        </is>
+      </c>
+      <c r="F24" s="9" t="inlineStr">
+        <is>
+          <t>https://github.com/shadps4-emu/shadPS4/releases
+https://github.com/shadps4-emu/shadps4-qtlauncher/releases</t>
+        </is>
+      </c>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>Veraltet: PS4 jetzt mit PS4 PKG Tool einrichten. Bestehende Installationen bleiben startbar; shadPS4 und QTLauncher werden im shadPS4 Manager des Tools verwaltet.</t>
+        </is>
+      </c>
+      <c r="H24" s="8" t="inlineStr">
+        <is>
+          <t>Veraltet: PS4 jetzt mit PS4 PKG Tool einrichten. Bestehende Installationen bleiben startbar; shadPS4 und QTLauncher werden im shadPS4 Manager des Tools verwaltet. Frühes Entwicklungsstadium und beschränkte Spielekompatibilität. Nur eigene Spiele verwenden; PKG-Dateien sind nicht direkt startbar. Vorübergehend im Hub ausgeblendet; mit Einstellungen → Ausgeblendete Einträge anzeigen wieder sichtbar. Bestehende Nutzerdaten bleiben erhalten.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="180" customHeight="1">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>Sony</t>
+        </is>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>PlayStation 4 (Hilfsprogramm)</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>PS4 PKG Tool</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>Windows (x64; .NET 10 Windows Desktop Runtime)</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>Niedrig</t>
+        </is>
+      </c>
+      <c r="F25" s="9" t="inlineStr">
+        <is>
+          <t>https://github.com/pearlxcore/PS4PKGTool/releases</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>PS4 einrichten lädt das Tool erst nach ausdrücklicher Bestätigung aus einem stabilen offiziellen Release. Bei installiertem Tool öffnet der Button dessen Hauptfenster. 1) PS4 PKG Tool über PS4 einrichten starten. 2) Tools &gt; shadPS4 Manager öffnen; shadPS4 über Install shadPS4 und QTLauncher installieren. 3) Im Manager den Spielebibliotheksordner festlegen. 4) Eigene PKG und passende Update-PKG laden; Install to shadPS4 wählen. 5) QTLauncher starten. Menünamen können sich in neuen Versionen ändern. Nur eigene Spiele verwenden.</t>
+        </is>
+      </c>
+      <c r="H25" s="8" t="inlineStr">
+        <is>
+          <t>Hilfsprogramm, kein Emulator. Der shadPS4 Manager des Tools übernimmt die Einrichtung von shadPS4 und QTLauncher. Nur eigene Spiele-PKGs; im Hub als Im PS4 PKG Tool installieren erfasst und nicht startbar. Der Hub öffnet das Tool oder übergibt einen Pfad an den Viewer. Keine eigene Entschlüsselung, Paketinstallation oder Schlüssel/Key-Dateien. Unabhängiges GPL-3.0-Drittprogramm, nicht mitgeliefert. Menünamen können sich ändern. Vorübergehend im Hub ausgeblendet; mit Einstellungen → Ausgeblendete Einträge anzeigen wieder sichtbar. Bestehende Nutzerdaten bleiben erhalten.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="300" customHeight="1">
+      <c r="A26" s="8" t="inlineStr">
+        <is>
+          <t>Commodore / Amiga</t>
+        </is>
+      </c>
+      <c r="B26" s="8" t="inlineStr">
+        <is>
+          <t>Amiga (A500, A1200, CD32 …)</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>WinUAE</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>Niedrig</t>
+        </is>
+      </c>
+      <c r="F26" s="9" t="inlineStr">
+        <is>
+          <t>WinUAE – offizielle Downloadseite</t>
+        </is>
+      </c>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>1. Die offizielle Downloadseite https://www.winuae.net/download/ öffnen und die aktuelle stabile Version im Abschnitt WinUAE prüfen. Beta-, Erweiterungs- und alte Downloads überspringen. 2. Im aktuellen Versionsabschnitt Download (64-bit) als ZIP wählen, nicht den MSI-Installer und nicht das 32-Bit-ZIP. Geprüft: WinUAE6030_x64.zip für 6.0.3, offiziell verlinkt unter https://download.abime.net/winuae/releases/. 3. Das vollständige ZIP in einen eigenen beschreibbaren Ordner entpacken. Geprüfte Startdatei: winuae64.exe. Den Ordner bei Bedarf über Ordner auswählen im Hub registrieren. 4. Ein eigenes lizenziertes oder selbst gesichertes Kickstart-ROM bereitstellen. In WinUAE unter Paths den ROMs-Ordner wählen und das zum Amiga-Modell passende Kickstart in der ROM-Auswahl einstellen. 5. Hardwaremodell und eigene Disk-/Festplatten-/CD-Abbilder in WinUAE passend konfigurieren; die Konfiguration als eigene .uae-Datei speichern. Images sind über WinUAE-Konfiguration zu starten; der Hub kann nur diese vorbereitete .uae-Konfiguration direkt laden. 6. Updates werden für automatische Installationen über die aktuelle stabile Version der offiziellen Downloadseite geprüft. Falls die Seite nicht eindeutig erkannt wird oder der Ordner manuell zugeordnet ist, die Version auf dieser Seite manuell prüfen.</t>
+        </is>
+      </c>
+      <c r="H26" s="8" t="inlineStr">
+        <is>
+          <t>WinUAE enthält kein Kickstart-ROM. Du brauchst ein lizenziertes bzw. aus eigener Amiga-Hardware selbst gesichertes Kickstart (z. B. gekauft mit Amiga Forever). Der Hub lädt, verlinkt oder bündelt keine Kickstart-ROMs, Spiele (ADF-Abbilder usw.) oder Workbench-Dateien. Eigene Images sind über WinUAE-Konfiguration zu starten; Hardwaremodell und benötigte eigene ROM-Dateien vorher in WinUAE einrichten.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="32" customHeight="1">
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>Hinweis: Switch bleibt außerhalb dieser Liste. shadPS4 für PlayStation 4 ist in einem frühen Entwicklungsstadium; die Spielekompatibilität ist beschränkt.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H23"/>
+  <autoFilter ref="A1:H26"/>
   <mergeCells count="1">
-    <mergeCell ref="A25:H25"/>
+    <mergeCell ref="A27:H27"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
@@ -1819,6 +1956,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F22" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F26" r:id="rId25"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>

</xml_diff>